<commit_message>
added second branch for processing and abel transforamrion
</commit_message>
<xml_diff>
--- a/abel_results_0.xlsx
+++ b/abel_results_0.xlsx
@@ -425,18 +425,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Radius_1</t>
+          <t>Radius_left_1</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Line_1</t>
+          <t>Line_left_1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Radius_right_1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Line_right_1</t>
         </is>
       </c>
     </row>
@@ -445,79 +455,139 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>12353.07597436099</v>
+        <v>230465.5721214064</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>257644.4047953101</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.4185</v>
+        <v>0.372</v>
       </c>
       <c r="B3" t="n">
-        <v>11909.93583816149</v>
+        <v>217851.1982372759</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.2945</v>
+      </c>
+      <c r="D3" t="n">
+        <v>252048.2794737096</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.837</v>
+        <v>0.7285</v>
       </c>
       <c r="B4" t="n">
-        <v>10673.23080926703</v>
+        <v>191385.0165612317</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.6045</v>
+      </c>
+      <c r="D4" t="n">
+        <v>225783.2723917807</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1.2555</v>
+        <v>1.085</v>
       </c>
       <c r="B5" t="n">
-        <v>8901.558960962137</v>
+        <v>157919.8751620956</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.9145</v>
+      </c>
+      <c r="D5" t="n">
+        <v>186539.5889852907</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1.674</v>
+        <v>1.457</v>
       </c>
       <c r="B6" t="n">
-        <v>6909.22900612222</v>
+        <v>115847.5020930622</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.2245</v>
+      </c>
+      <c r="D6" t="n">
+        <v>142386.098170912</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2.0925</v>
+        <v>1.8135</v>
       </c>
       <c r="B7" t="n">
-        <v>4993.188750173028</v>
+        <v>79884.16187273385</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.5345</v>
+      </c>
+      <c r="D7" t="n">
+        <v>100498.9257493175</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2.511</v>
+        <v>2.17</v>
       </c>
       <c r="B8" t="n">
-        <v>3363.779227733827</v>
+        <v>51806.79887178875</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.8445</v>
+      </c>
+      <c r="D8" t="n">
+        <v>65668.99685320635</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2.9295</v>
+        <v>2.542</v>
       </c>
       <c r="B9" t="n">
-        <v>2118.61440993345</v>
+        <v>29736.94288760151</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2.1545</v>
+      </c>
+      <c r="D9" t="n">
+        <v>39839.84389480402</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3.348</v>
+        <v>2.8985</v>
       </c>
       <c r="B10" t="n">
-        <v>1252.692406857509</v>
+        <v>16105.26182403005</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2.4645</v>
+      </c>
+      <c r="D10" t="n">
+        <v>22308.05498067966</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3.782</v>
+        <v>3.255</v>
       </c>
       <c r="B11" t="n">
-        <v>868.7912517867333</v>
+        <v>10335.5537502479</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2.7745</v>
+      </c>
+      <c r="D11" t="n">
+        <v>14873.37671938059</v>
       </c>
     </row>
   </sheetData>

</xml_diff>